<commit_message>
seperating things and furthering FF work
</commit_message>
<xml_diff>
--- a/spreadsheets/03_MAD/M0111A/M0111A.xlsx
+++ b/spreadsheets/03_MAD/M0111A/M0111A.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e255fabf6a46c9b0/Desktop/Work stuff/SURF 2026/MAD-FF-Corrections-from-Varied-Salinity/spreadsheets/03_MAD/M0111A/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="11_9C7812B6000284D3929A09BD5B3BF2B185EEE75F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7910D2E5-F0F5-4EF1-BBED-418E557872ED}"/>
+  <xr:revisionPtr revIDLastSave="5" documentId="11_9C7812B6000284D3929A09BD5B3BF2B185EEE75F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2FD7ED82-60F9-412D-B3E4-2BC4872EB5A5}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -13446,19 +13446,19 @@
         <v>1.5117098445595856</v>
       </c>
       <c r="Y2" s="20">
-        <f t="shared" ref="Y2:Y26" si="5">X2-(V2-W2)</f>
+        <f>X2-(V2-W2)</f>
         <v>5.2909844559585473E-2</v>
       </c>
       <c r="Z2" s="20">
-        <f t="shared" ref="Z2:Z26" si="6">W2-Y2</f>
+        <f t="shared" ref="Z2:Z26" si="5">W2-Y2</f>
         <v>7.6087901554404143</v>
       </c>
       <c r="AA2" s="20">
-        <f t="shared" ref="AA2:AA26" si="7">X2/1.024</f>
+        <f t="shared" ref="AA2:AA26" si="6">X2/1.024</f>
         <v>1.4762791450777202</v>
       </c>
       <c r="AB2" s="20">
-        <f t="shared" ref="AB2:AB26" si="8">Y2/2.22</f>
+        <f t="shared" ref="AB2:AB26" si="7">Y2/2.22</f>
         <v>2.383326331512859E-2</v>
       </c>
       <c r="AC2" s="20">
@@ -13466,39 +13466,39 @@
         <v>2.8785773094170395</v>
       </c>
       <c r="AD2" s="20">
-        <f t="shared" ref="AD2:AD26" si="9">AC2-AB2+AA2</f>
+        <f t="shared" ref="AD2:AD26" si="8">AC2-AB2+AA2</f>
         <v>4.3310231911796313</v>
       </c>
       <c r="AE2" s="20">
-        <f t="shared" ref="AE2:AE26" si="10">AC2-AB2</f>
+        <f t="shared" ref="AE2:AE26" si="9">AC2-AB2</f>
         <v>2.8547440461019109</v>
       </c>
       <c r="AF2" s="20">
-        <f t="shared" ref="AF2:AF26" si="11">X2/V2</f>
+        <f t="shared" ref="AF2:AF26" si="10">X2/V2</f>
         <v>0.16574857130196652</v>
       </c>
       <c r="AG2" s="20">
-        <f t="shared" ref="AG2:AG26" si="12">X2/Z2</f>
+        <f t="shared" ref="AG2:AG26" si="11">X2/Z2</f>
         <v>0.19867939760156053</v>
       </c>
       <c r="AH2" s="20">
-        <f t="shared" ref="AH2:AH26" si="13">V2/AD2</f>
+        <f t="shared" ref="AH2:AH26" si="12">V2/AD2</f>
         <v>2.1058534201743373</v>
       </c>
       <c r="AI2" s="20">
-        <f t="shared" ref="AI2:AI26" si="14">Z2/AD2</f>
+        <f t="shared" ref="AI2:AI26" si="13">Z2/AD2</f>
         <v>1.7568112244090812</v>
       </c>
       <c r="AJ2" s="20">
-        <f t="shared" ref="AJ2:AJ26" si="15">Z2/AE2</f>
+        <f t="shared" ref="AJ2:AJ26" si="14">Z2/AE2</f>
         <v>2.6653143092915972</v>
       </c>
       <c r="AK2" s="20">
-        <f t="shared" ref="AK2:AK26" si="16">AA2/AD2</f>
+        <f t="shared" ref="AK2:AK26" si="15">AA2/AD2</f>
         <v>0.34086151930200798</v>
       </c>
       <c r="AL2" s="20">
-        <f t="shared" ref="AL2:AL26" si="17">AA2/AE2</f>
+        <f t="shared" ref="AL2:AL26" si="16">AA2/AE2</f>
         <v>0.51713187635632218</v>
       </c>
     </row>
@@ -13570,7 +13570,7 @@
       </c>
       <c r="U3" s="22"/>
       <c r="V3" s="20">
-        <f t="shared" ref="V2:V26" si="18">O3-N3</f>
+        <f t="shared" ref="V2:V26" si="17">O3-N3</f>
         <v>9.953400000000002</v>
       </c>
       <c r="W3" s="20">
@@ -13582,19 +13582,19 @@
         <v>2.0139896373056998</v>
       </c>
       <c r="Y3" s="20">
+        <f t="shared" ref="Y2:Y26" si="18">X3-(V3-W3)</f>
+        <v>7.0489637305699571E-2</v>
+      </c>
+      <c r="Z3" s="20">
         <f t="shared" si="5"/>
-        <v>7.0489637305699571E-2</v>
-      </c>
-      <c r="Z3" s="20">
+        <v>7.9394103626943018</v>
+      </c>
+      <c r="AA3" s="20">
         <f t="shared" si="6"/>
-        <v>7.9394103626943018</v>
-      </c>
-      <c r="AA3" s="20">
+        <v>1.9667867551813474</v>
+      </c>
+      <c r="AB3" s="20">
         <f t="shared" si="7"/>
-        <v>1.9667867551813474</v>
-      </c>
-      <c r="AB3" s="20">
-        <f t="shared" si="8"/>
         <v>3.1752088876441244E-2</v>
       </c>
       <c r="AC3" s="20">
@@ -13602,39 +13602,39 @@
         <v>3.0170677130044794</v>
       </c>
       <c r="AD3" s="20">
+        <f t="shared" si="8"/>
+        <v>4.9521023793093857</v>
+      </c>
+      <c r="AE3" s="20">
         <f t="shared" si="9"/>
-        <v>4.9521023793093857</v>
-      </c>
-      <c r="AE3" s="20">
+        <v>2.9853156241280381</v>
+      </c>
+      <c r="AF3" s="20">
         <f t="shared" si="10"/>
-        <v>2.9853156241280381</v>
-      </c>
-      <c r="AF3" s="20">
+        <v>0.2023418768768159</v>
+      </c>
+      <c r="AG3" s="20">
         <f t="shared" si="11"/>
-        <v>0.2023418768768159</v>
-      </c>
-      <c r="AG3" s="20">
+        <v>0.2536699257628795</v>
+      </c>
+      <c r="AH3" s="20">
         <f t="shared" si="12"/>
-        <v>0.2536699257628795</v>
-      </c>
-      <c r="AH3" s="20">
+        <v>2.0099342133124662</v>
+      </c>
+      <c r="AI3" s="20">
         <f t="shared" si="13"/>
-        <v>2.0099342133124662</v>
-      </c>
-      <c r="AI3" s="20">
+        <v>1.6032403521918952</v>
+      </c>
+      <c r="AJ3" s="20">
         <f t="shared" si="14"/>
-        <v>1.6032403521918952</v>
-      </c>
-      <c r="AJ3" s="20">
+        <v>2.6594877601973073</v>
+      </c>
+      <c r="AK3" s="20">
         <f t="shared" si="15"/>
-        <v>2.6594877601973073</v>
-      </c>
-      <c r="AK3" s="20">
+        <v>0.39716197375055745</v>
+      </c>
+      <c r="AL3" s="20">
         <f t="shared" si="16"/>
-        <v>0.39716197375055745</v>
-      </c>
-      <c r="AL3" s="20">
-        <f t="shared" si="17"/>
         <v>0.65882037372708746</v>
       </c>
     </row>
@@ -13705,7 +13705,7 @@
         <v>7.2446000000000002</v>
       </c>
       <c r="V4" s="20">
-        <f t="shared" si="18"/>
+        <f t="shared" si="17"/>
         <v>8.8712</v>
       </c>
       <c r="W4" s="20">
@@ -13717,19 +13717,19 @@
         <v>1.7589637305699464</v>
       </c>
       <c r="Y4" s="20">
+        <f t="shared" si="18"/>
+        <v>6.1563730569948127E-2</v>
+      </c>
+      <c r="Z4" s="20">
         <f t="shared" si="5"/>
-        <v>6.1563730569948127E-2</v>
-      </c>
-      <c r="Z4" s="20">
+        <v>7.1122362694300536</v>
+      </c>
+      <c r="AA4" s="20">
         <f t="shared" si="6"/>
-        <v>7.1122362694300536</v>
-      </c>
-      <c r="AA4" s="20">
+        <v>1.7177380181347133</v>
+      </c>
+      <c r="AB4" s="20">
         <f t="shared" si="7"/>
-        <v>1.7177380181347133</v>
-      </c>
-      <c r="AB4" s="20">
-        <f t="shared" si="8"/>
         <v>2.7731410166643298E-2</v>
       </c>
       <c r="AC4" s="20">
@@ -13737,39 +13737,39 @@
         <v>2.7120439461883405</v>
       </c>
       <c r="AD4" s="20">
+        <f t="shared" si="8"/>
+        <v>4.4020505541564106</v>
+      </c>
+      <c r="AE4" s="20">
         <f t="shared" si="9"/>
-        <v>4.4020505541564106</v>
-      </c>
-      <c r="AE4" s="20">
+        <v>2.6843125360216971</v>
+      </c>
+      <c r="AF4" s="20">
         <f t="shared" si="10"/>
-        <v>2.6843125360216971</v>
-      </c>
-      <c r="AF4" s="20">
+        <v>0.19827799289497997</v>
+      </c>
+      <c r="AG4" s="20">
         <f t="shared" si="11"/>
-        <v>0.19827799289497997</v>
-      </c>
-      <c r="AG4" s="20">
+        <v>0.2473151430767784</v>
+      </c>
+      <c r="AH4" s="20">
         <f t="shared" si="12"/>
-        <v>0.2473151430767784</v>
-      </c>
-      <c r="AH4" s="20">
+        <v>2.0152426445043492</v>
+      </c>
+      <c r="AI4" s="20">
         <f t="shared" si="13"/>
-        <v>2.0152426445043492</v>
-      </c>
-      <c r="AI4" s="20">
+        <v>1.615664377755655</v>
+      </c>
+      <c r="AJ4" s="20">
         <f t="shared" si="14"/>
-        <v>1.615664377755655</v>
-      </c>
-      <c r="AJ4" s="20">
+        <v>2.6495559566885567</v>
+      </c>
+      <c r="AK4" s="20">
         <f t="shared" si="15"/>
-        <v>2.6495559566885567</v>
-      </c>
-      <c r="AK4" s="20">
+        <v>0.39021315112177146</v>
+      </c>
+      <c r="AL4" s="20">
         <f t="shared" si="16"/>
-        <v>0.39021315112177146</v>
-      </c>
-      <c r="AL4" s="20">
-        <f t="shared" si="17"/>
         <v>0.63991729542808684</v>
       </c>
     </row>
@@ -13840,7 +13840,7 @@
         <v>7.2667000000000002</v>
       </c>
       <c r="V5" s="20">
-        <f t="shared" si="18"/>
+        <f t="shared" si="17"/>
         <v>9.7160999999999991</v>
       </c>
       <c r="W5" s="20">
@@ -13852,19 +13852,19 @@
         <v>1.9311917098445577</v>
       </c>
       <c r="Y5" s="20">
+        <f t="shared" si="18"/>
+        <v>6.7591709844559533E-2</v>
+      </c>
+      <c r="Z5" s="20">
         <f t="shared" si="5"/>
-        <v>6.7591709844559533E-2</v>
-      </c>
-      <c r="Z5" s="20">
+        <v>7.7849082901554416</v>
+      </c>
+      <c r="AA5" s="20">
         <f t="shared" si="6"/>
-        <v>7.7849082901554416</v>
-      </c>
-      <c r="AA5" s="20">
+        <v>1.8859294041450758</v>
+      </c>
+      <c r="AB5" s="20">
         <f t="shared" si="7"/>
-        <v>1.8859294041450758</v>
-      </c>
-      <c r="AB5" s="20">
-        <f t="shared" si="8"/>
         <v>3.0446716146197986E-2</v>
       </c>
       <c r="AC5" s="20">
@@ -13872,39 +13872,39 @@
         <v>2.9392560538116603</v>
       </c>
       <c r="AD5" s="20">
+        <f t="shared" si="8"/>
+        <v>4.7947387418105381</v>
+      </c>
+      <c r="AE5" s="20">
         <f t="shared" si="9"/>
-        <v>4.7947387418105381</v>
-      </c>
-      <c r="AE5" s="20">
+        <v>2.9088093376654625</v>
+      </c>
+      <c r="AF5" s="20">
         <f t="shared" si="10"/>
-        <v>2.9088093376654625</v>
-      </c>
-      <c r="AF5" s="20">
+        <v>0.19876202487053013</v>
+      </c>
+      <c r="AG5" s="20">
         <f t="shared" si="11"/>
-        <v>0.19876202487053013</v>
-      </c>
-      <c r="AG5" s="20">
+        <v>0.24806865256032418</v>
+      </c>
+      <c r="AH5" s="20">
         <f t="shared" si="12"/>
-        <v>0.24806865256032418</v>
-      </c>
-      <c r="AH5" s="20">
+        <v>2.0264086372996224</v>
+      </c>
+      <c r="AI5" s="20">
         <f t="shared" si="13"/>
-        <v>2.0264086372996224</v>
-      </c>
-      <c r="AI5" s="20">
+        <v>1.6236355533348179</v>
+      </c>
+      <c r="AJ5" s="20">
         <f t="shared" si="14"/>
-        <v>1.6236355533348179</v>
-      </c>
-      <c r="AJ5" s="20">
+        <v>2.6763212663513429</v>
+      </c>
+      <c r="AK5" s="20">
         <f t="shared" si="15"/>
-        <v>2.6763212663513429</v>
-      </c>
-      <c r="AK5" s="20">
+        <v>0.39333308980937953</v>
+      </c>
+      <c r="AL5" s="20">
         <f t="shared" si="16"/>
-        <v>0.39333308980937953</v>
-      </c>
-      <c r="AL5" s="20">
-        <f t="shared" si="17"/>
         <v>0.64835098668195135</v>
       </c>
     </row>
@@ -13975,7 +13975,7 @@
         <v>7.1943999999999999</v>
       </c>
       <c r="V6" s="20">
-        <f t="shared" si="18"/>
+        <f t="shared" si="17"/>
         <v>8.7312999999999992</v>
       </c>
       <c r="W6" s="20">
@@ -13987,19 +13987,19 @@
         <v>1.6031088082901561</v>
       </c>
       <c r="Y6" s="20">
+        <f t="shared" si="18"/>
+        <v>5.6108808290155521E-2</v>
+      </c>
+      <c r="Z6" s="20">
         <f t="shared" si="5"/>
-        <v>5.6108808290155521E-2</v>
-      </c>
-      <c r="Z6" s="20">
+        <v>7.1281911917098428</v>
+      </c>
+      <c r="AA6" s="20">
         <f t="shared" si="6"/>
-        <v>7.1281911917098428</v>
-      </c>
-      <c r="AA6" s="20">
+        <v>1.5655359455958555</v>
+      </c>
+      <c r="AB6" s="20">
         <f t="shared" si="7"/>
-        <v>1.5655359455958555</v>
-      </c>
-      <c r="AB6" s="20">
-        <f t="shared" si="8"/>
         <v>2.5274237968538522E-2</v>
       </c>
       <c r="AC6" s="20">
@@ -14007,39 +14007,39 @@
         <v>2.6852071748878901</v>
       </c>
       <c r="AD6" s="20">
+        <f t="shared" si="8"/>
+        <v>4.2254688825152069</v>
+      </c>
+      <c r="AE6" s="20">
         <f t="shared" si="9"/>
-        <v>4.2254688825152069</v>
-      </c>
-      <c r="AE6" s="20">
+        <v>2.6599329369193514</v>
+      </c>
+      <c r="AF6" s="20">
         <f t="shared" si="10"/>
-        <v>2.6599329369193514</v>
-      </c>
-      <c r="AF6" s="20">
+        <v>0.18360482497338956</v>
+      </c>
+      <c r="AG6" s="20">
         <f t="shared" si="11"/>
-        <v>0.18360482497338956</v>
-      </c>
-      <c r="AG6" s="20">
+        <v>0.22489699913697428</v>
+      </c>
+      <c r="AH6" s="20">
         <f t="shared" si="12"/>
-        <v>0.22489699913697428</v>
-      </c>
-      <c r="AH6" s="20">
+        <v>2.0663505619766154</v>
+      </c>
+      <c r="AI6" s="20">
         <f t="shared" si="13"/>
-        <v>2.0663505619766154</v>
-      </c>
-      <c r="AI6" s="20">
+        <v>1.6869586287112337</v>
+      </c>
+      <c r="AJ6" s="20">
         <f t="shared" si="14"/>
-        <v>1.6869586287112337</v>
-      </c>
-      <c r="AJ6" s="20">
+        <v>2.6798386879503378</v>
+      </c>
+      <c r="AK6" s="20">
         <f t="shared" si="15"/>
-        <v>2.6798386879503378</v>
-      </c>
-      <c r="AK6" s="20">
+        <v>0.37049993482947424</v>
+      </c>
+      <c r="AL6" s="20">
         <f t="shared" si="16"/>
-        <v>0.37049993482947424</v>
-      </c>
-      <c r="AL6" s="20">
-        <f t="shared" si="17"/>
         <v>0.58856218661249737</v>
       </c>
     </row>
@@ -14110,7 +14110,7 @@
         <v>7.5315000000000003</v>
       </c>
       <c r="V7" s="20">
-        <f t="shared" si="18"/>
+        <f t="shared" si="17"/>
         <v>10.022599999999999</v>
       </c>
       <c r="W7" s="20">
@@ -14122,19 +14122,19 @@
         <v>2.0734715025906714</v>
       </c>
       <c r="Y7" s="20">
+        <f t="shared" si="18"/>
+        <v>7.2571502590673465E-2</v>
+      </c>
+      <c r="Z7" s="20">
         <f t="shared" si="5"/>
-        <v>7.2571502590673465E-2</v>
-      </c>
-      <c r="Z7" s="20">
+        <v>7.9491284974093279</v>
+      </c>
+      <c r="AA7" s="20">
         <f t="shared" si="6"/>
-        <v>7.9491284974093279</v>
-      </c>
-      <c r="AA7" s="20">
+        <v>2.0248745142487024</v>
+      </c>
+      <c r="AB7" s="20">
         <f t="shared" si="7"/>
-        <v>2.0248745142487024</v>
-      </c>
-      <c r="AB7" s="20">
-        <f t="shared" si="8"/>
         <v>3.2689866031834894E-2</v>
       </c>
       <c r="AC7" s="20">
@@ -14142,39 +14142,39 @@
         <v>3.0243251121076202</v>
       </c>
       <c r="AD7" s="20">
+        <f t="shared" si="8"/>
+        <v>5.016509760324487</v>
+      </c>
+      <c r="AE7" s="20">
         <f t="shared" si="9"/>
-        <v>5.016509760324487</v>
-      </c>
-      <c r="AE7" s="20">
+        <v>2.9916352460757851</v>
+      </c>
+      <c r="AF7" s="20">
         <f t="shared" si="10"/>
-        <v>2.9916352460757851</v>
-      </c>
-      <c r="AF7" s="20">
+        <v>0.20687960235773867</v>
+      </c>
+      <c r="AG7" s="20">
         <f t="shared" si="11"/>
-        <v>0.20687960235773867</v>
-      </c>
-      <c r="AG7" s="20">
+        <v>0.26084261982510776</v>
+      </c>
+      <c r="AH7" s="20">
         <f t="shared" si="12"/>
-        <v>0.26084261982510776</v>
-      </c>
-      <c r="AH7" s="20">
+        <v>1.9979229541759524</v>
+      </c>
+      <c r="AI7" s="20">
         <f t="shared" si="13"/>
-        <v>1.9979229541759524</v>
-      </c>
-      <c r="AI7" s="20">
+        <v>1.5845934478746331</v>
+      </c>
+      <c r="AJ7" s="20">
         <f t="shared" si="14"/>
-        <v>1.5845934478746331</v>
-      </c>
-      <c r="AJ7" s="20">
+        <v>2.6571182124680575</v>
+      </c>
+      <c r="AK7" s="20">
         <f t="shared" si="15"/>
-        <v>2.6571182124680575</v>
-      </c>
-      <c r="AK7" s="20">
+        <v>0.40364209599738238</v>
+      </c>
+      <c r="AL7" s="20">
         <f t="shared" si="16"/>
-        <v>0.40364209599738238</v>
-      </c>
-      <c r="AL7" s="20">
-        <f t="shared" si="17"/>
         <v>0.67684538645036663</v>
       </c>
     </row>
@@ -14245,7 +14245,7 @@
         <v>6.5564</v>
       </c>
       <c r="V8" s="20">
-        <f t="shared" si="18"/>
+        <f t="shared" si="17"/>
         <v>7.4625000000000004</v>
       </c>
       <c r="W8" s="20">
@@ -14257,19 +14257,19 @@
         <v>1.4433160621761671</v>
       </c>
       <c r="Y8" s="20">
+        <f t="shared" si="18"/>
+        <v>5.0516062176165999E-2</v>
+      </c>
+      <c r="Z8" s="20">
         <f t="shared" si="5"/>
-        <v>5.0516062176165999E-2</v>
-      </c>
-      <c r="Z8" s="20">
+        <v>6.0191839378238328</v>
+      </c>
+      <c r="AA8" s="20">
         <f t="shared" si="6"/>
-        <v>6.0191839378238328</v>
-      </c>
-      <c r="AA8" s="20">
+        <v>1.4094883419689133</v>
+      </c>
+      <c r="AB8" s="20">
         <f t="shared" si="7"/>
-        <v>1.4094883419689133</v>
-      </c>
-      <c r="AB8" s="20">
-        <f t="shared" si="8"/>
         <v>2.2754982962236936E-2</v>
       </c>
       <c r="AC8" s="20">
@@ -14277,39 +14277,39 @@
         <v>2.2742026905829604</v>
       </c>
       <c r="AD8" s="20">
+        <f t="shared" si="8"/>
+        <v>3.6609360495896368</v>
+      </c>
+      <c r="AE8" s="20">
         <f t="shared" si="9"/>
-        <v>3.6609360495896368</v>
-      </c>
-      <c r="AE8" s="20">
+        <v>2.2514477076207235</v>
+      </c>
+      <c r="AF8" s="20">
         <f t="shared" si="10"/>
-        <v>2.2514477076207235</v>
-      </c>
-      <c r="AF8" s="20">
+        <v>0.19340918756129541</v>
+      </c>
+      <c r="AG8" s="20">
         <f t="shared" si="11"/>
-        <v>0.19340918756129541</v>
-      </c>
-      <c r="AG8" s="20">
+        <v>0.23978600373159248</v>
+      </c>
+      <c r="AH8" s="20">
         <f t="shared" si="12"/>
-        <v>0.23978600373159248</v>
-      </c>
-      <c r="AH8" s="20">
+        <v>2.0384130995231371</v>
+      </c>
+      <c r="AI8" s="20">
         <f t="shared" si="13"/>
-        <v>2.0384130995231371</v>
-      </c>
-      <c r="AI8" s="20">
+        <v>1.6441652780300648</v>
+      </c>
+      <c r="AJ8" s="20">
         <f t="shared" si="14"/>
-        <v>1.6441652780300648</v>
-      </c>
-      <c r="AJ8" s="20">
+        <v>2.6734726804669</v>
+      </c>
+      <c r="AK8" s="20">
         <f t="shared" si="15"/>
-        <v>2.6734726804669</v>
-      </c>
-      <c r="AK8" s="20">
+        <v>0.38500763817682809</v>
+      </c>
+      <c r="AL8" s="20">
         <f t="shared" si="16"/>
-        <v>0.38500763817682809</v>
-      </c>
-      <c r="AL8" s="20">
-        <f t="shared" si="17"/>
         <v>0.62603645520971352</v>
       </c>
     </row>
@@ -14380,7 +14380,7 @@
         <v>7.0872999999999999</v>
       </c>
       <c r="V9" s="20">
-        <f t="shared" si="18"/>
+        <f t="shared" si="17"/>
         <v>8.2801000000000009</v>
       </c>
       <c r="W9" s="20">
@@ -14392,19 +14392,19 @@
         <v>1.6578238341968932</v>
       </c>
       <c r="Y9" s="20">
+        <f t="shared" si="18"/>
+        <v>5.8023834196891277E-2</v>
+      </c>
+      <c r="Z9" s="20">
         <f t="shared" si="5"/>
-        <v>5.8023834196891277E-2</v>
-      </c>
-      <c r="Z9" s="20">
+        <v>6.6222761658031075</v>
+      </c>
+      <c r="AA9" s="20">
         <f t="shared" si="6"/>
-        <v>6.6222761658031075</v>
-      </c>
-      <c r="AA9" s="20">
+        <v>1.6189685880829034</v>
+      </c>
+      <c r="AB9" s="20">
         <f t="shared" si="7"/>
-        <v>1.6189685880829034</v>
-      </c>
-      <c r="AB9" s="20">
-        <f t="shared" si="8"/>
         <v>2.6136862250851923E-2</v>
       </c>
       <c r="AC9" s="20">
@@ -14412,39 +14412,39 @@
         <v>2.5272103139013398</v>
       </c>
       <c r="AD9" s="20">
+        <f t="shared" si="8"/>
+        <v>4.1200420397333914</v>
+      </c>
+      <c r="AE9" s="20">
         <f t="shared" si="9"/>
-        <v>4.1200420397333914</v>
-      </c>
-      <c r="AE9" s="20">
+        <v>2.501073451650488</v>
+      </c>
+      <c r="AF9" s="20">
         <f t="shared" si="10"/>
-        <v>2.501073451650488</v>
-      </c>
-      <c r="AF9" s="20">
+        <v>0.20021785174054577</v>
+      </c>
+      <c r="AG9" s="20">
         <f t="shared" si="11"/>
-        <v>0.20021785174054577</v>
-      </c>
-      <c r="AG9" s="20">
+        <v>0.25034048606395487</v>
+      </c>
+      <c r="AH9" s="20">
         <f t="shared" si="12"/>
-        <v>0.25034048606395487</v>
-      </c>
-      <c r="AH9" s="20">
+        <v>2.0097125029665492</v>
+      </c>
+      <c r="AI9" s="20">
         <f t="shared" si="13"/>
-        <v>2.0097125029665492</v>
-      </c>
-      <c r="AI9" s="20">
+        <v>1.6073321830064715</v>
+      </c>
+      <c r="AJ9" s="20">
         <f t="shared" si="14"/>
-        <v>1.6073321830064715</v>
-      </c>
-      <c r="AJ9" s="20">
+        <v>2.6477735635604742</v>
+      </c>
+      <c r="AK9" s="20">
         <f t="shared" si="15"/>
-        <v>2.6477735635604742</v>
-      </c>
-      <c r="AK9" s="20">
+        <v>0.39294953121101334</v>
+      </c>
+      <c r="AL9" s="20">
         <f t="shared" si="16"/>
-        <v>0.39294953121101334</v>
-      </c>
-      <c r="AL9" s="20">
-        <f t="shared" si="17"/>
         <v>0.64730949305568253</v>
       </c>
       <c r="AN9" s="8">
@@ -14519,7 +14519,7 @@
         <v>7.9097999999999997</v>
       </c>
       <c r="V10" s="20">
-        <f t="shared" si="18"/>
+        <f t="shared" si="17"/>
         <v>10.625599999999999</v>
       </c>
       <c r="W10" s="20">
@@ -14531,19 +14531,19 @@
         <v>1.8404145077720206</v>
       </c>
       <c r="Y10" s="20">
+        <f t="shared" si="18"/>
+        <v>6.4414507772020846E-2</v>
+      </c>
+      <c r="Z10" s="20">
         <f t="shared" si="5"/>
-        <v>6.4414507772020846E-2</v>
-      </c>
-      <c r="Z10" s="20">
+        <v>8.7851854922279777</v>
+      </c>
+      <c r="AA10" s="20">
         <f t="shared" si="6"/>
-        <v>8.7851854922279777</v>
-      </c>
-      <c r="AA10" s="20">
+        <v>1.7972797927461139</v>
+      </c>
+      <c r="AB10" s="20">
         <f t="shared" si="7"/>
-        <v>1.7972797927461139</v>
-      </c>
-      <c r="AB10" s="20">
-        <f t="shared" si="8"/>
         <v>2.901554404145083E-2</v>
       </c>
       <c r="AC10" s="20">
@@ -14551,39 +14551,39 @@
         <v>3.3536565022421501</v>
       </c>
       <c r="AD10" s="20">
+        <f t="shared" si="8"/>
+        <v>5.1219207509468134</v>
+      </c>
+      <c r="AE10" s="20">
         <f t="shared" si="9"/>
-        <v>5.1219207509468134</v>
-      </c>
-      <c r="AE10" s="20">
+        <v>3.3246409582006993</v>
+      </c>
+      <c r="AF10" s="20">
         <f t="shared" si="10"/>
-        <v>3.3246409582006993</v>
-      </c>
-      <c r="AF10" s="20">
+        <v>0.17320570205654465</v>
+      </c>
+      <c r="AG10" s="20">
         <f t="shared" si="11"/>
-        <v>0.17320570205654465</v>
-      </c>
-      <c r="AG10" s="20">
+        <v>0.20949068285469749</v>
+      </c>
+      <c r="AH10" s="20">
         <f t="shared" si="12"/>
-        <v>0.20949068285469749</v>
-      </c>
-      <c r="AH10" s="20">
+        <v>2.0745342453874946</v>
+      </c>
+      <c r="AI10" s="20">
         <f t="shared" si="13"/>
-        <v>2.0745342453874946</v>
-      </c>
-      <c r="AI10" s="20">
+        <v>1.7152130849748097</v>
+      </c>
+      <c r="AJ10" s="20">
         <f t="shared" si="14"/>
-        <v>1.7152130849748097</v>
-      </c>
-      <c r="AJ10" s="20">
+        <v>2.6424463882507583</v>
+      </c>
+      <c r="AK10" s="20">
         <f t="shared" si="15"/>
-        <v>2.6424463882507583</v>
-      </c>
-      <c r="AK10" s="20">
+        <v>0.35089957071551281</v>
+      </c>
+      <c r="AL10" s="20">
         <f t="shared" si="16"/>
-        <v>0.35089957071551281</v>
-      </c>
-      <c r="AL10" s="20">
-        <f t="shared" si="17"/>
         <v>0.54059365066560583</v>
       </c>
     </row>
@@ -14654,7 +14654,7 @@
         <v>7.9249000000000001</v>
       </c>
       <c r="V11" s="20">
-        <f t="shared" si="18"/>
+        <f t="shared" si="17"/>
         <v>11.302</v>
       </c>
       <c r="W11" s="20">
@@ -14666,19 +14666,19 @@
         <v>1.8189637305699464</v>
       </c>
       <c r="Y11" s="20">
+        <f t="shared" si="18"/>
+        <v>6.3663730569948118E-2</v>
+      </c>
+      <c r="Z11" s="20">
         <f t="shared" si="5"/>
-        <v>6.3663730569948118E-2</v>
-      </c>
-      <c r="Z11" s="20">
+        <v>9.4830362694300536</v>
+      </c>
+      <c r="AA11" s="20">
         <f t="shared" si="6"/>
-        <v>9.4830362694300536</v>
-      </c>
-      <c r="AA11" s="20">
+        <v>1.7763317681347133</v>
+      </c>
+      <c r="AB11" s="20">
         <f t="shared" si="7"/>
-        <v>1.7763317681347133</v>
-      </c>
-      <c r="AB11" s="20">
-        <f t="shared" si="8"/>
         <v>2.8677356112589241E-2</v>
       </c>
       <c r="AC11" s="20">
@@ -14686,39 +14686,39 @@
         <v>3.5793394618834098</v>
       </c>
       <c r="AD11" s="20">
+        <f t="shared" si="8"/>
+        <v>5.3269938739055336</v>
+      </c>
+      <c r="AE11" s="20">
         <f t="shared" si="9"/>
-        <v>5.3269938739055336</v>
-      </c>
-      <c r="AE11" s="20">
+        <v>3.5506621057708205</v>
+      </c>
+      <c r="AF11" s="20">
         <f t="shared" si="10"/>
-        <v>3.5506621057708205</v>
-      </c>
-      <c r="AF11" s="20">
+        <v>0.16094175637674274</v>
+      </c>
+      <c r="AG11" s="20">
         <f t="shared" si="11"/>
-        <v>0.16094175637674274</v>
-      </c>
-      <c r="AG11" s="20">
+        <v>0.19181237726925504</v>
+      </c>
+      <c r="AH11" s="20">
         <f t="shared" si="12"/>
-        <v>0.19181237726925504</v>
-      </c>
-      <c r="AH11" s="20">
+        <v>2.1216468926993222</v>
+      </c>
+      <c r="AI11" s="20">
         <f t="shared" si="13"/>
-        <v>2.1216468926993222</v>
-      </c>
-      <c r="AI11" s="20">
+        <v>1.7801853153770346</v>
+      </c>
+      <c r="AJ11" s="20">
         <f t="shared" si="14"/>
-        <v>1.7801853153770346</v>
-      </c>
-      <c r="AJ11" s="20">
+        <v>2.6707796988109522</v>
+      </c>
+      <c r="AK11" s="20">
         <f t="shared" si="15"/>
-        <v>2.6707796988109522</v>
-      </c>
-      <c r="AK11" s="20">
+        <v>0.33345857160379644</v>
+      </c>
+      <c r="AL11" s="20">
         <f t="shared" si="16"/>
-        <v>0.33345857160379644</v>
-      </c>
-      <c r="AL11" s="20">
-        <f t="shared" si="17"/>
         <v>0.5002818390540954</v>
       </c>
     </row>
@@ -14789,7 +14789,7 @@
         <v>7.2873000000000001</v>
       </c>
       <c r="V12" s="20">
-        <f t="shared" si="18"/>
+        <f t="shared" si="17"/>
         <v>9.3326000000000011</v>
       </c>
       <c r="W12" s="20">
@@ -14801,19 +14801,19 @@
         <v>1.6189637305699487</v>
       </c>
       <c r="Y12" s="20">
+        <f t="shared" si="18"/>
+        <v>5.6663730569948223E-2</v>
+      </c>
+      <c r="Z12" s="20">
         <f t="shared" si="5"/>
-        <v>5.6663730569948223E-2</v>
-      </c>
-      <c r="Z12" s="20">
+        <v>7.7136362694300526</v>
+      </c>
+      <c r="AA12" s="20">
         <f t="shared" si="6"/>
-        <v>7.7136362694300526</v>
-      </c>
-      <c r="AA12" s="20">
+        <v>1.5810192681347155</v>
+      </c>
+      <c r="AB12" s="20">
         <f t="shared" si="7"/>
-        <v>1.5810192681347155</v>
-      </c>
-      <c r="AB12" s="20">
-        <f t="shared" si="8"/>
         <v>2.5524202959436134E-2</v>
       </c>
       <c r="AC12" s="20">
@@ -14821,39 +14821,39 @@
         <v>2.9237125560538102</v>
       </c>
       <c r="AD12" s="20">
+        <f t="shared" si="8"/>
+        <v>4.4792076212290892</v>
+      </c>
+      <c r="AE12" s="20">
         <f t="shared" si="9"/>
-        <v>4.4792076212290892</v>
-      </c>
-      <c r="AE12" s="20">
+        <v>2.8981883530943739</v>
+      </c>
+      <c r="AF12" s="20">
         <f t="shared" si="10"/>
-        <v>2.8981883530943739</v>
-      </c>
-      <c r="AF12" s="20">
+        <v>0.17347402980626497</v>
+      </c>
+      <c r="AG12" s="20">
         <f t="shared" si="11"/>
-        <v>0.17347402980626497</v>
-      </c>
-      <c r="AG12" s="20">
+        <v>0.20988333828833378</v>
+      </c>
+      <c r="AH12" s="20">
         <f t="shared" si="12"/>
-        <v>0.20988333828833378</v>
-      </c>
-      <c r="AH12" s="20">
+        <v>2.083538158795851</v>
+      </c>
+      <c r="AI12" s="20">
         <f t="shared" si="13"/>
-        <v>2.083538158795851</v>
-      </c>
-      <c r="AI12" s="20">
+        <v>1.7220983981344093</v>
+      </c>
+      <c r="AJ12" s="20">
         <f t="shared" si="14"/>
-        <v>1.7220983981344093</v>
-      </c>
-      <c r="AJ12" s="20">
+        <v>2.6615372535033002</v>
+      </c>
+      <c r="AK12" s="20">
         <f t="shared" si="15"/>
-        <v>2.6615372535033002</v>
-      </c>
-      <c r="AK12" s="20">
+        <v>0.35296851627093939</v>
+      </c>
+      <c r="AL12" s="20">
         <f t="shared" si="16"/>
-        <v>0.35296851627093939</v>
-      </c>
-      <c r="AL12" s="20">
-        <f t="shared" si="17"/>
         <v>0.54551984740628512</v>
       </c>
     </row>
@@ -14924,7 +14924,7 @@
         <v>8.1348000000000003</v>
       </c>
       <c r="V13" s="20">
-        <f t="shared" si="18"/>
+        <f t="shared" si="17"/>
         <v>12.486999999999998</v>
       </c>
       <c r="W13" s="20">
@@ -14936,19 +14936,19 @@
         <v>2.7473575129533674</v>
       </c>
       <c r="Y13" s="20">
+        <f t="shared" si="18"/>
+        <v>9.6157512953368052E-2</v>
+      </c>
+      <c r="Z13" s="20">
         <f t="shared" si="5"/>
-        <v>9.6157512953368052E-2</v>
-      </c>
-      <c r="Z13" s="20">
+        <v>9.7396424870466305</v>
+      </c>
+      <c r="AA13" s="20">
         <f t="shared" si="6"/>
-        <v>9.7396424870466305</v>
-      </c>
-      <c r="AA13" s="20">
+        <v>2.6829663212435229</v>
+      </c>
+      <c r="AB13" s="20">
         <f t="shared" si="7"/>
-        <v>2.6829663212435229</v>
-      </c>
-      <c r="AB13" s="20">
-        <f t="shared" si="8"/>
         <v>4.3314195024039659E-2</v>
       </c>
       <c r="AC13" s="20">
@@ -14956,39 +14956,39 @@
         <v>3.6902708520179406</v>
       </c>
       <c r="AD13" s="20">
+        <f t="shared" si="8"/>
+        <v>6.3299229782374233</v>
+      </c>
+      <c r="AE13" s="20">
         <f t="shared" si="9"/>
-        <v>6.3299229782374233</v>
-      </c>
-      <c r="AE13" s="20">
+        <v>3.6469566569939009</v>
+      </c>
+      <c r="AF13" s="20">
         <f t="shared" si="10"/>
-        <v>3.6469566569939009</v>
-      </c>
-      <c r="AF13" s="20">
+        <v>0.2200174191521877</v>
+      </c>
+      <c r="AG13" s="20">
         <f t="shared" si="11"/>
-        <v>0.2200174191521877</v>
-      </c>
-      <c r="AG13" s="20">
+        <v>0.28207991377581393</v>
+      </c>
+      <c r="AH13" s="20">
         <f t="shared" si="12"/>
-        <v>0.28207991377581393</v>
-      </c>
-      <c r="AH13" s="20">
+        <v>1.9726938294400893</v>
+      </c>
+      <c r="AI13" s="20">
         <f t="shared" si="13"/>
-        <v>1.9726938294400893</v>
-      </c>
-      <c r="AI13" s="20">
+        <v>1.538666824309235</v>
+      </c>
+      <c r="AJ13" s="20">
         <f t="shared" si="14"/>
-        <v>1.538666824309235</v>
-      </c>
-      <c r="AJ13" s="20">
+        <v>2.6706219467589682</v>
+      </c>
+      <c r="AK13" s="20">
         <f t="shared" si="15"/>
-        <v>2.6706219467589682</v>
-      </c>
-      <c r="AK13" s="20">
+        <v>0.42385449719810003</v>
+      </c>
+      <c r="AL13" s="20">
         <f t="shared" si="16"/>
-        <v>0.42385449719810003</v>
-      </c>
-      <c r="AL13" s="20">
-        <f t="shared" si="17"/>
         <v>0.73567266452106062</v>
       </c>
     </row>
@@ -15059,7 +15059,7 @@
         <v>7.2150999999999996</v>
       </c>
       <c r="V14" s="20">
-        <f t="shared" si="18"/>
+        <f t="shared" si="17"/>
         <v>8.8401999999999994</v>
       </c>
       <c r="W14" s="20">
@@ -15071,19 +15071,19 @@
         <v>1.6678756476683907</v>
       </c>
       <c r="Y14" s="20">
+        <f t="shared" si="18"/>
+        <v>5.8375647668393649E-2</v>
+      </c>
+      <c r="Z14" s="20">
         <f t="shared" si="5"/>
-        <v>5.8375647668393649E-2</v>
-      </c>
-      <c r="Z14" s="20">
+        <v>7.1723243523316089</v>
+      </c>
+      <c r="AA14" s="20">
         <f t="shared" si="6"/>
-        <v>7.1723243523316089</v>
-      </c>
-      <c r="AA14" s="20">
+        <v>1.6287848121761628</v>
+      </c>
+      <c r="AB14" s="20">
         <f t="shared" si="7"/>
-        <v>1.6287848121761628</v>
-      </c>
-      <c r="AB14" s="20">
-        <f t="shared" si="8"/>
         <v>2.6295336787564703E-2</v>
       </c>
       <c r="AC14" s="20">
@@ -15091,39 +15091,39 @@
         <v>2.6889565022421493</v>
       </c>
       <c r="AD14" s="20">
+        <f t="shared" si="8"/>
+        <v>4.2914459776307474</v>
+      </c>
+      <c r="AE14" s="20">
         <f t="shared" si="9"/>
-        <v>4.2914459776307474</v>
-      </c>
-      <c r="AE14" s="20">
+        <v>2.6626611654545846</v>
+      </c>
+      <c r="AF14" s="20">
         <f t="shared" si="10"/>
-        <v>2.6626611654545846</v>
-      </c>
-      <c r="AF14" s="20">
+        <v>0.18866944726006096</v>
+      </c>
+      <c r="AG14" s="20">
         <f t="shared" si="11"/>
-        <v>0.18866944726006096</v>
-      </c>
-      <c r="AG14" s="20">
+        <v>0.23254325456240565</v>
+      </c>
+      <c r="AH14" s="20">
         <f t="shared" si="12"/>
-        <v>0.23254325456240565</v>
-      </c>
-      <c r="AH14" s="20">
+        <v>2.0599583557802492</v>
+      </c>
+      <c r="AI14" s="20">
         <f t="shared" si="13"/>
-        <v>2.0599583557802492</v>
-      </c>
-      <c r="AI14" s="20">
+        <v>1.6713071514164459</v>
+      </c>
+      <c r="AJ14" s="20">
         <f t="shared" si="14"/>
-        <v>1.6713071514164459</v>
-      </c>
-      <c r="AJ14" s="20">
+        <v>2.6936676905741814</v>
+      </c>
+      <c r="AK14" s="20">
         <f t="shared" si="15"/>
-        <v>2.6936676905741814</v>
-      </c>
-      <c r="AK14" s="20">
+        <v>0.37954219176152698</v>
+      </c>
+      <c r="AL14" s="20">
         <f t="shared" si="16"/>
-        <v>0.37954219176152698</v>
-      </c>
-      <c r="AL14" s="20">
-        <f t="shared" si="17"/>
         <v>0.61171313620675705</v>
       </c>
     </row>
@@ -15194,7 +15194,7 @@
         <v>7.1925999999999997</v>
       </c>
       <c r="V15" s="20">
-        <f t="shared" si="18"/>
+        <f t="shared" si="17"/>
         <v>9.1006999999999998</v>
       </c>
       <c r="W15" s="20">
@@ -15206,19 +15206,19 @@
         <v>1.5586528497409338</v>
       </c>
       <c r="Y15" s="20">
+        <f t="shared" si="18"/>
+        <v>5.4552849740932663E-2</v>
+      </c>
+      <c r="Z15" s="20">
         <f t="shared" si="5"/>
-        <v>5.4552849740932663E-2</v>
-      </c>
-      <c r="Z15" s="20">
+        <v>7.5420471502590658</v>
+      </c>
+      <c r="AA15" s="20">
         <f t="shared" si="6"/>
-        <v>7.5420471502590658</v>
-      </c>
-      <c r="AA15" s="20">
+        <v>1.5221219235751307</v>
+      </c>
+      <c r="AB15" s="20">
         <f t="shared" si="7"/>
-        <v>1.5221219235751307</v>
-      </c>
-      <c r="AB15" s="20">
-        <f t="shared" si="8"/>
         <v>2.4573355739158854E-2</v>
       </c>
       <c r="AC15" s="20">
@@ -15226,39 +15226,39 @@
         <v>2.8683847533632294</v>
       </c>
       <c r="AD15" s="20">
+        <f t="shared" si="8"/>
+        <v>4.3659333211992015</v>
+      </c>
+      <c r="AE15" s="20">
         <f t="shared" si="9"/>
-        <v>4.3659333211992015</v>
-      </c>
-      <c r="AE15" s="20">
+        <v>2.8438113976240706</v>
+      </c>
+      <c r="AF15" s="20">
         <f t="shared" si="10"/>
-        <v>2.8438113976240706</v>
-      </c>
-      <c r="AF15" s="20">
+        <v>0.17126735852636982</v>
+      </c>
+      <c r="AG15" s="20">
         <f t="shared" si="11"/>
-        <v>0.17126735852636982</v>
-      </c>
-      <c r="AG15" s="20">
+        <v>0.20666177480571635</v>
+      </c>
+      <c r="AH15" s="20">
         <f t="shared" si="12"/>
-        <v>0.20666177480571635</v>
-      </c>
-      <c r="AH15" s="20">
+        <v>2.0844798421017314</v>
+      </c>
+      <c r="AI15" s="20">
         <f t="shared" si="13"/>
-        <v>2.0844798421017314</v>
-      </c>
-      <c r="AI15" s="20">
+        <v>1.7274764856435034</v>
+      </c>
+      <c r="AJ15" s="20">
         <f t="shared" si="14"/>
-        <v>1.7274764856435034</v>
-      </c>
-      <c r="AJ15" s="20">
+        <v>2.6520911888039578</v>
+      </c>
+      <c r="AK15" s="20">
         <f t="shared" si="15"/>
-        <v>2.6520911888039578</v>
-      </c>
-      <c r="AK15" s="20">
+        <v>0.34863609029123827</v>
+      </c>
+      <c r="AL15" s="20">
         <f t="shared" si="16"/>
-        <v>0.34863609029123827</v>
-      </c>
-      <c r="AL15" s="20">
-        <f t="shared" si="17"/>
         <v>0.53524010939924616</v>
       </c>
     </row>
@@ -15329,7 +15329,7 @@
         <v>7.6210000000000004</v>
       </c>
       <c r="V16" s="20">
-        <f t="shared" si="18"/>
+        <f t="shared" si="17"/>
         <v>10.2377</v>
       </c>
       <c r="W16" s="20">
@@ -15341,19 +15341,19 @@
         <v>2.0029015544041453</v>
       </c>
       <c r="Y16" s="20">
+        <f t="shared" si="18"/>
+        <v>7.0101554404145006E-2</v>
+      </c>
+      <c r="Z16" s="20">
         <f t="shared" si="5"/>
-        <v>7.0101554404145006E-2</v>
-      </c>
-      <c r="Z16" s="20">
+        <v>8.2347984455958549</v>
+      </c>
+      <c r="AA16" s="20">
         <f t="shared" si="6"/>
-        <v>8.2347984455958549</v>
-      </c>
-      <c r="AA16" s="20">
+        <v>1.9559585492227982</v>
+      </c>
+      <c r="AB16" s="20">
         <f t="shared" si="7"/>
-        <v>1.9559585492227982</v>
-      </c>
-      <c r="AB16" s="20">
-        <f t="shared" si="8"/>
         <v>3.1577276758623873E-2</v>
       </c>
       <c r="AC16" s="20">
@@ -15361,39 +15361,39 @@
         <v>3.1775470852017902</v>
       </c>
       <c r="AD16" s="20">
+        <f t="shared" si="8"/>
+        <v>5.1019283576659644</v>
+      </c>
+      <c r="AE16" s="20">
         <f t="shared" si="9"/>
-        <v>5.1019283576659644</v>
-      </c>
-      <c r="AE16" s="20">
+        <v>3.1459698084431662</v>
+      </c>
+      <c r="AF16" s="20">
         <f t="shared" si="10"/>
-        <v>3.1459698084431662</v>
-      </c>
-      <c r="AF16" s="20">
+        <v>0.19563979745491128</v>
+      </c>
+      <c r="AG16" s="20">
         <f t="shared" si="11"/>
-        <v>0.19563979745491128</v>
-      </c>
-      <c r="AG16" s="20">
+        <v>0.24322411381851605</v>
+      </c>
+      <c r="AH16" s="20">
         <f t="shared" si="12"/>
-        <v>0.24322411381851605</v>
-      </c>
-      <c r="AH16" s="20">
+        <v>2.0066334300083262</v>
+      </c>
+      <c r="AI16" s="20">
         <f t="shared" si="13"/>
-        <v>2.0066334300083262</v>
-      </c>
-      <c r="AI16" s="20">
+        <v>1.6140560721952433</v>
+      </c>
+      <c r="AJ16" s="20">
         <f t="shared" si="14"/>
-        <v>1.6140560721952433</v>
-      </c>
-      <c r="AJ16" s="20">
+        <v>2.6175707165069642</v>
+      </c>
+      <c r="AK16" s="20">
         <f t="shared" si="15"/>
-        <v>2.6175707165069642</v>
-      </c>
-      <c r="AK16" s="20">
+        <v>0.38337632598933868</v>
+      </c>
+      <c r="AL16" s="20">
         <f t="shared" si="16"/>
-        <v>0.38337632598933868</v>
-      </c>
-      <c r="AL16" s="20">
-        <f t="shared" si="17"/>
         <v>0.62173468542939891</v>
       </c>
     </row>
@@ -15464,7 +15464,7 @@
         <v>7.7865000000000002</v>
       </c>
       <c r="V17" s="20">
-        <f t="shared" si="18"/>
+        <f t="shared" si="17"/>
         <v>11.039899999999999</v>
       </c>
       <c r="W17" s="20">
@@ -15476,19 +15476,19 @@
         <v>2.7018652849740921</v>
       </c>
       <c r="Y17" s="20">
+        <f t="shared" si="18"/>
+        <v>9.4565284974093444E-2</v>
+      </c>
+      <c r="Z17" s="20">
         <f t="shared" si="5"/>
-        <v>9.4565284974093444E-2</v>
-      </c>
-      <c r="Z17" s="20">
+        <v>8.3380347150259073</v>
+      </c>
+      <c r="AA17" s="20">
         <f t="shared" si="6"/>
-        <v>8.3380347150259073</v>
-      </c>
-      <c r="AA17" s="20">
+        <v>2.6385403173575117</v>
+      </c>
+      <c r="AB17" s="20">
         <f t="shared" si="7"/>
-        <v>2.6385403173575117</v>
-      </c>
-      <c r="AB17" s="20">
-        <f t="shared" si="8"/>
         <v>4.2596975213555599E-2</v>
       </c>
       <c r="AC17" s="20">
@@ -15496,39 +15496,39 @@
         <v>3.4067242152466406</v>
       </c>
       <c r="AD17" s="20">
+        <f t="shared" si="8"/>
+        <v>6.0026675573905965</v>
+      </c>
+      <c r="AE17" s="20">
         <f t="shared" si="9"/>
-        <v>6.0026675573905965</v>
-      </c>
-      <c r="AE17" s="20">
+        <v>3.3641272400330848</v>
+      </c>
+      <c r="AF17" s="20">
         <f t="shared" si="10"/>
-        <v>3.3641272400330848</v>
-      </c>
-      <c r="AF17" s="20">
+        <v>0.2447363911787328</v>
+      </c>
+      <c r="AG17" s="20">
         <f t="shared" si="11"/>
-        <v>0.2447363911787328</v>
-      </c>
-      <c r="AG17" s="20">
+        <v>0.32404102133384999</v>
+      </c>
+      <c r="AH17" s="20">
         <f t="shared" si="12"/>
-        <v>0.32404102133384999</v>
-      </c>
-      <c r="AH17" s="20">
+        <v>1.8391656533448146</v>
+      </c>
+      <c r="AI17" s="20">
         <f t="shared" si="13"/>
-        <v>1.8391656533448146</v>
-      </c>
-      <c r="AI17" s="20">
+        <v>1.3890548885653284</v>
+      </c>
+      <c r="AJ17" s="20">
         <f t="shared" si="14"/>
-        <v>1.3890548885653284</v>
-      </c>
-      <c r="AJ17" s="20">
+        <v>2.4785134806446578</v>
+      </c>
+      <c r="AK17" s="20">
         <f t="shared" si="15"/>
-        <v>2.4785134806446578</v>
-      </c>
-      <c r="AK17" s="20">
+        <v>0.43956129372996705</v>
+      </c>
+      <c r="AL17" s="20">
         <f t="shared" si="16"/>
-        <v>0.43956129372996705</v>
-      </c>
-      <c r="AL17" s="20">
-        <f t="shared" si="17"/>
         <v>0.78431644497833042</v>
       </c>
     </row>
@@ -15599,7 +15599,7 @@
         <v>7.5921000000000003</v>
       </c>
       <c r="V18" s="20">
-        <f t="shared" si="18"/>
+        <f t="shared" si="17"/>
         <v>10.042499999999999</v>
       </c>
       <c r="W18" s="20">
@@ -15611,19 +15611,19 @@
         <v>1.7780310880828996</v>
       </c>
       <c r="Y18" s="20">
+        <f t="shared" si="18"/>
+        <v>6.2231088082901564E-2</v>
+      </c>
+      <c r="Z18" s="20">
         <f t="shared" si="5"/>
-        <v>6.2231088082901564E-2</v>
-      </c>
-      <c r="Z18" s="20">
+        <v>8.2644689119170991</v>
+      </c>
+      <c r="AA18" s="20">
         <f t="shared" si="6"/>
-        <v>8.2644689119170991</v>
-      </c>
-      <c r="AA18" s="20">
+        <v>1.7363584844559565</v>
+      </c>
+      <c r="AB18" s="20">
         <f t="shared" si="7"/>
-        <v>1.7363584844559565</v>
-      </c>
-      <c r="AB18" s="20">
-        <f t="shared" si="8"/>
         <v>2.8032021658964665E-2</v>
       </c>
       <c r="AC18" s="20">
@@ -15631,39 +15631,39 @@
         <v>3.1444318385650201</v>
       </c>
       <c r="AD18" s="20">
+        <f t="shared" si="8"/>
+        <v>4.8527583013620124</v>
+      </c>
+      <c r="AE18" s="20">
         <f t="shared" si="9"/>
-        <v>4.8527583013620124</v>
-      </c>
-      <c r="AE18" s="20">
+        <v>3.1163998169060556</v>
+      </c>
+      <c r="AF18" s="20">
         <f t="shared" si="10"/>
-        <v>3.1163998169060556</v>
-      </c>
-      <c r="AF18" s="20">
+        <v>0.17705064357310429</v>
+      </c>
+      <c r="AG18" s="20">
         <f t="shared" si="11"/>
-        <v>0.17705064357310429</v>
-      </c>
-      <c r="AG18" s="20">
+        <v>0.21514160280995623</v>
+      </c>
+      <c r="AH18" s="20">
         <f t="shared" si="12"/>
-        <v>0.21514160280995623</v>
-      </c>
-      <c r="AH18" s="20">
+        <v>2.0694416198683117</v>
+      </c>
+      <c r="AI18" s="20">
         <f t="shared" si="13"/>
-        <v>2.0694416198683117</v>
-      </c>
-      <c r="AI18" s="20">
+        <v>1.7030456492336594</v>
+      </c>
+      <c r="AJ18" s="20">
         <f t="shared" si="14"/>
-        <v>1.7030456492336594</v>
-      </c>
-      <c r="AJ18" s="20">
+        <v>2.6519283139099969</v>
+      </c>
+      <c r="AK18" s="20">
         <f t="shared" si="15"/>
-        <v>2.6519283139099969</v>
-      </c>
-      <c r="AK18" s="20">
+        <v>0.35780856507290232</v>
+      </c>
+      <c r="AL18" s="20">
         <f t="shared" si="16"/>
-        <v>0.35780856507290232</v>
-      </c>
-      <c r="AL18" s="20">
-        <f t="shared" si="17"/>
         <v>0.55716807421064596</v>
       </c>
     </row>
@@ -15734,7 +15734,7 @@
         <v>8.2136999999999993</v>
       </c>
       <c r="V19" s="20">
-        <f t="shared" si="18"/>
+        <f t="shared" si="17"/>
         <v>11.930999999999999</v>
       </c>
       <c r="W19" s="20">
@@ -15746,19 +15746,19 @@
         <v>2.0112953367875641</v>
       </c>
       <c r="Y19" s="20">
+        <f t="shared" si="18"/>
+        <v>7.0395336787564933E-2</v>
+      </c>
+      <c r="Z19" s="20">
         <f t="shared" si="5"/>
-        <v>7.0395336787564933E-2</v>
-      </c>
-      <c r="Z19" s="20">
+        <v>9.9197046632124355</v>
+      </c>
+      <c r="AA19" s="20">
         <f t="shared" si="6"/>
-        <v>9.9197046632124355</v>
-      </c>
-      <c r="AA19" s="20">
+        <v>1.9641556023316056</v>
+      </c>
+      <c r="AB19" s="20">
         <f t="shared" si="7"/>
-        <v>1.9641556023316056</v>
-      </c>
-      <c r="AB19" s="20">
-        <f t="shared" si="8"/>
         <v>3.1709611165569786E-2</v>
       </c>
       <c r="AC19" s="20">
@@ -15766,39 +15766,39 @@
         <v>3.7898434977578495</v>
       </c>
       <c r="AD19" s="20">
+        <f t="shared" si="8"/>
+        <v>5.7222894889238853</v>
+      </c>
+      <c r="AE19" s="20">
         <f t="shared" si="9"/>
-        <v>5.7222894889238853</v>
-      </c>
-      <c r="AE19" s="20">
+        <v>3.7581338865922795</v>
+      </c>
+      <c r="AF19" s="20">
         <f t="shared" si="10"/>
-        <v>3.7581338865922795</v>
-      </c>
-      <c r="AF19" s="20">
+        <v>0.16857726400029874</v>
+      </c>
+      <c r="AG19" s="20">
         <f t="shared" si="11"/>
-        <v>0.16857726400029874</v>
-      </c>
-      <c r="AG19" s="20">
+        <v>0.20275758251619341</v>
+      </c>
+      <c r="AH19" s="20">
         <f t="shared" si="12"/>
-        <v>0.20275758251619341</v>
-      </c>
-      <c r="AH19" s="20">
+        <v>2.0850046162630798</v>
+      </c>
+      <c r="AI19" s="20">
         <f t="shared" si="13"/>
-        <v>2.0850046162630798</v>
-      </c>
-      <c r="AI19" s="20">
+        <v>1.733520242625457</v>
+      </c>
+      <c r="AJ19" s="20">
         <f t="shared" si="14"/>
-        <v>1.733520242625457</v>
-      </c>
-      <c r="AJ19" s="20">
+        <v>2.6395293415709609</v>
+      </c>
+      <c r="AK19" s="20">
         <f t="shared" si="15"/>
-        <v>2.6395293415709609</v>
-      </c>
-      <c r="AK19" s="20">
+        <v>0.34324645863049097</v>
+      </c>
+      <c r="AL19" s="20">
         <f t="shared" si="16"/>
-        <v>0.34324645863049097</v>
-      </c>
-      <c r="AL19" s="20">
-        <f t="shared" si="17"/>
         <v>0.5226411994897342</v>
       </c>
     </row>
@@ -15869,7 +15869,7 @@
         <v>8.1577000000000002</v>
       </c>
       <c r="V20" s="20">
-        <f t="shared" si="18"/>
+        <f t="shared" si="17"/>
         <v>12.1326</v>
       </c>
       <c r="W20" s="20">
@@ -15881,19 +15881,19 @@
         <v>2.6205181347150264</v>
       </c>
       <c r="Y20" s="20">
+        <f t="shared" si="18"/>
+        <v>9.171813471502599E-2</v>
+      </c>
+      <c r="Z20" s="20">
         <f t="shared" si="5"/>
-        <v>9.171813471502599E-2</v>
-      </c>
-      <c r="Z20" s="20">
+        <v>9.5120818652849728</v>
+      </c>
+      <c r="AA20" s="20">
         <f t="shared" si="6"/>
-        <v>9.5120818652849728</v>
-      </c>
-      <c r="AA20" s="20">
+        <v>2.559099740932643</v>
+      </c>
+      <c r="AB20" s="20">
         <f t="shared" si="7"/>
-        <v>2.559099740932643</v>
-      </c>
-      <c r="AB20" s="20">
-        <f t="shared" si="8"/>
         <v>4.1314475096858552E-2</v>
       </c>
       <c r="AC20" s="20">
@@ -15901,39 +15901,39 @@
         <v>3.6029914798206306</v>
       </c>
       <c r="AD20" s="20">
+        <f t="shared" si="8"/>
+        <v>6.1207767456564151</v>
+      </c>
+      <c r="AE20" s="20">
         <f t="shared" si="9"/>
-        <v>6.1207767456564151</v>
-      </c>
-      <c r="AE20" s="20">
+        <v>3.561677004723772</v>
+      </c>
+      <c r="AF20" s="20">
         <f t="shared" si="10"/>
-        <v>3.561677004723772</v>
-      </c>
-      <c r="AF20" s="20">
+        <v>0.21598982367464734</v>
+      </c>
+      <c r="AG20" s="20">
         <f t="shared" si="11"/>
-        <v>0.21598982367464734</v>
-      </c>
-      <c r="AG20" s="20">
+        <v>0.27549364816537125</v>
+      </c>
+      <c r="AH20" s="20">
         <f t="shared" si="12"/>
-        <v>0.27549364816537125</v>
-      </c>
-      <c r="AH20" s="20">
+        <v>1.982199401180553</v>
+      </c>
+      <c r="AI20" s="20">
         <f t="shared" si="13"/>
-        <v>1.982199401180553</v>
-      </c>
-      <c r="AI20" s="20">
+        <v>1.5540645020315738</v>
+      </c>
+      <c r="AJ20" s="20">
         <f t="shared" si="14"/>
-        <v>1.5540645020315738</v>
-      </c>
-      <c r="AJ20" s="20">
+        <v>2.6706750366945999</v>
+      </c>
+      <c r="AK20" s="20">
         <f t="shared" si="15"/>
-        <v>2.6706750366945999</v>
-      </c>
-      <c r="AK20" s="20">
+        <v>0.41810048745017503</v>
+      </c>
+      <c r="AL20" s="20">
         <f t="shared" si="16"/>
-        <v>0.41810048745017503</v>
-      </c>
-      <c r="AL20" s="20">
-        <f t="shared" si="17"/>
         <v>0.71850977433904495</v>
       </c>
     </row>
@@ -16004,7 +16004,7 @@
         <v>7.3446999999999996</v>
       </c>
       <c r="V21" s="20">
-        <f t="shared" si="18"/>
+        <f t="shared" si="17"/>
         <v>9.8346</v>
       </c>
       <c r="W21" s="20">
@@ -16016,19 +16016,19 @@
         <v>2.2887046632124357</v>
       </c>
       <c r="Y21" s="20">
+        <f t="shared" si="18"/>
+        <v>8.0104663212435145E-2</v>
+      </c>
+      <c r="Z21" s="20">
         <f t="shared" si="5"/>
-        <v>8.0104663212435145E-2</v>
-      </c>
-      <c r="Z21" s="20">
+        <v>7.5458953367875647</v>
+      </c>
+      <c r="AA21" s="20">
         <f t="shared" si="6"/>
-        <v>7.5458953367875647</v>
-      </c>
-      <c r="AA21" s="20">
+        <v>2.2350631476683942</v>
+      </c>
+      <c r="AB21" s="20">
         <f t="shared" si="7"/>
-        <v>2.2350631476683942</v>
-      </c>
-      <c r="AB21" s="20">
-        <f t="shared" si="8"/>
         <v>3.6083181627223036E-2</v>
       </c>
       <c r="AC21" s="20">
@@ -16036,39 +16036,39 @@
         <v>2.8690946188340796</v>
       </c>
       <c r="AD21" s="20">
+        <f t="shared" si="8"/>
+        <v>5.0680745848752506</v>
+      </c>
+      <c r="AE21" s="20">
         <f t="shared" si="9"/>
-        <v>5.0680745848752506</v>
-      </c>
-      <c r="AE21" s="20">
+        <v>2.8330114372068564</v>
+      </c>
+      <c r="AF21" s="20">
         <f t="shared" si="10"/>
-        <v>2.8330114372068564</v>
-      </c>
-      <c r="AF21" s="20">
+        <v>0.23271964932101313</v>
+      </c>
+      <c r="AG21" s="20">
         <f t="shared" si="11"/>
-        <v>0.23271964932101313</v>
-      </c>
-      <c r="AG21" s="20">
+        <v>0.30330458627680651</v>
+      </c>
+      <c r="AH21" s="20">
         <f t="shared" si="12"/>
-        <v>0.30330458627680651</v>
-      </c>
-      <c r="AH21" s="20">
+        <v>1.9405002502034165</v>
+      </c>
+      <c r="AI21" s="20">
         <f t="shared" si="13"/>
-        <v>1.9405002502034165</v>
-      </c>
-      <c r="AI21" s="20">
+        <v>1.4889077124687393</v>
+      </c>
+      <c r="AJ21" s="20">
         <f t="shared" si="14"/>
-        <v>1.4889077124687393</v>
-      </c>
-      <c r="AJ21" s="20">
+        <v>2.663559785775969</v>
+      </c>
+      <c r="AK21" s="20">
         <f t="shared" si="15"/>
-        <v>2.663559785775969</v>
-      </c>
-      <c r="AK21" s="20">
+        <v>0.44100833763152081</v>
+      </c>
+      <c r="AL21" s="20">
         <f t="shared" si="16"/>
-        <v>0.44100833763152081</v>
-      </c>
-      <c r="AL21" s="20">
-        <f t="shared" si="17"/>
         <v>0.78893544809406213</v>
       </c>
     </row>
@@ -16139,7 +16139,7 @@
         <v>7.4241000000000001</v>
       </c>
       <c r="V22" s="20">
-        <f t="shared" si="18"/>
+        <f t="shared" si="17"/>
         <v>10.3911</v>
       </c>
       <c r="W22" s="20">
@@ -16151,19 +16151,19 @@
         <v>2.1756476683937813</v>
       </c>
       <c r="Y22" s="20">
+        <f t="shared" si="18"/>
+        <v>7.6147668393782286E-2</v>
+      </c>
+      <c r="Z22" s="20">
         <f t="shared" si="5"/>
-        <v>7.6147668393782286E-2</v>
-      </c>
-      <c r="Z22" s="20">
+        <v>8.2154523316062189</v>
+      </c>
+      <c r="AA22" s="20">
         <f t="shared" si="6"/>
-        <v>8.2154523316062189</v>
-      </c>
-      <c r="AA22" s="20">
+        <v>2.124655926165802</v>
+      </c>
+      <c r="AB22" s="20">
         <f t="shared" si="7"/>
-        <v>2.124655926165802</v>
-      </c>
-      <c r="AB22" s="20">
-        <f t="shared" si="8"/>
         <v>3.4300751528730758E-2</v>
       </c>
       <c r="AC22" s="20">
@@ -16171,39 +16171,39 @@
         <v>3.1055798206278</v>
       </c>
       <c r="AD22" s="20">
+        <f t="shared" si="8"/>
+        <v>5.1959349952648708</v>
+      </c>
+      <c r="AE22" s="20">
         <f t="shared" si="9"/>
-        <v>5.1959349952648708</v>
-      </c>
-      <c r="AE22" s="20">
+        <v>3.0712790690990692</v>
+      </c>
+      <c r="AF22" s="20">
         <f t="shared" si="10"/>
-        <v>3.0712790690990692</v>
-      </c>
-      <c r="AF22" s="20">
+        <v>0.20937606878903883</v>
+      </c>
+      <c r="AG22" s="20">
         <f t="shared" si="11"/>
-        <v>0.20937606878903883</v>
-      </c>
-      <c r="AG22" s="20">
+        <v>0.26482384421168154</v>
+      </c>
+      <c r="AH22" s="20">
         <f t="shared" si="12"/>
-        <v>0.26482384421168154</v>
-      </c>
-      <c r="AH22" s="20">
+        <v>1.9998518090525683</v>
+      </c>
+      <c r="AI22" s="20">
         <f t="shared" si="13"/>
-        <v>1.9998518090525683</v>
-      </c>
-      <c r="AI22" s="20">
+        <v>1.581130699112494</v>
+      </c>
+      <c r="AJ22" s="20">
         <f t="shared" si="14"/>
-        <v>1.581130699112494</v>
-      </c>
-      <c r="AJ22" s="20">
+        <v>2.6749286361711651</v>
+      </c>
+      <c r="AK22" s="20">
         <f t="shared" si="15"/>
-        <v>2.6749286361711651</v>
-      </c>
-      <c r="AK22" s="20">
+        <v>0.40890733392585377</v>
+      </c>
+      <c r="AL22" s="20">
         <f t="shared" si="16"/>
-        <v>0.40890733392585377</v>
-      </c>
-      <c r="AL22" s="20">
-        <f t="shared" si="17"/>
         <v>0.69178211369410003</v>
       </c>
     </row>
@@ -16274,7 +16274,7 @@
         <v>7.6078000000000001</v>
       </c>
       <c r="V23" s="20">
-        <f t="shared" si="18"/>
+        <f t="shared" si="17"/>
         <v>10.47</v>
       </c>
       <c r="W23" s="20">
@@ -16286,19 +16286,19 @@
         <v>1.8917098445595872</v>
       </c>
       <c r="Y23" s="20">
+        <f t="shared" si="18"/>
+        <v>6.6209844559585562E-2</v>
+      </c>
+      <c r="Z23" s="20">
         <f t="shared" si="5"/>
-        <v>6.6209844559585562E-2</v>
-      </c>
-      <c r="Z23" s="20">
+        <v>8.5782901554404134</v>
+      </c>
+      <c r="AA23" s="20">
         <f t="shared" si="6"/>
-        <v>8.5782901554404134</v>
-      </c>
-      <c r="AA23" s="20">
+        <v>1.847372895077722</v>
+      </c>
+      <c r="AB23" s="20">
         <f t="shared" si="7"/>
-        <v>1.847372895077722</v>
-      </c>
-      <c r="AB23" s="20">
-        <f t="shared" si="8"/>
         <v>2.9824254306119621E-2</v>
       </c>
       <c r="AC23" s="20">
@@ -16306,39 +16306,39 @@
         <v>3.2338986547085202</v>
       </c>
       <c r="AD23" s="20">
+        <f t="shared" si="8"/>
+        <v>5.0514472954801226</v>
+      </c>
+      <c r="AE23" s="20">
         <f t="shared" si="9"/>
-        <v>5.0514472954801226</v>
-      </c>
-      <c r="AE23" s="20">
+        <v>3.2040744004024004</v>
+      </c>
+      <c r="AF23" s="20">
         <f t="shared" si="10"/>
-        <v>3.2040744004024004</v>
-      </c>
-      <c r="AF23" s="20">
+        <v>0.18067906824828911</v>
+      </c>
+      <c r="AG23" s="20">
         <f t="shared" si="11"/>
-        <v>0.18067906824828911</v>
-      </c>
-      <c r="AG23" s="20">
+        <v>0.2205229492452935</v>
+      </c>
+      <c r="AH23" s="20">
         <f t="shared" si="12"/>
-        <v>0.2205229492452935</v>
-      </c>
-      <c r="AH23" s="20">
+        <v>2.0726733127292509</v>
+      </c>
+      <c r="AI23" s="20">
         <f t="shared" si="13"/>
-        <v>2.0726733127292509</v>
-      </c>
-      <c r="AI23" s="20">
+        <v>1.6981846298022349</v>
+      </c>
+      <c r="AJ23" s="20">
         <f t="shared" si="14"/>
-        <v>1.6981846298022349</v>
-      </c>
-      <c r="AJ23" s="20">
+        <v>2.6773067923650786</v>
+      </c>
+      <c r="AK23" s="20">
         <f t="shared" si="15"/>
-        <v>2.6773067923650786</v>
-      </c>
-      <c r="AK23" s="20">
+        <v>0.36571160442091388</v>
+      </c>
+      <c r="AL23" s="20">
         <f t="shared" si="16"/>
-        <v>0.36571160442091388</v>
-      </c>
-      <c r="AL23" s="20">
-        <f t="shared" si="17"/>
         <v>0.5765699119988319</v>
       </c>
     </row>
@@ -16409,7 +16409,7 @@
         <v>7.4650999999999996</v>
       </c>
       <c r="V24" s="20">
-        <f t="shared" si="18"/>
+        <f t="shared" si="17"/>
         <v>9.984</v>
       </c>
       <c r="W24" s="20">
@@ -16421,19 +16421,19 @@
         <v>2.0744041450777195</v>
       </c>
       <c r="Y24" s="20">
+        <f t="shared" si="18"/>
+        <v>7.2604145077720172E-2</v>
+      </c>
+      <c r="Z24" s="20">
         <f t="shared" si="5"/>
-        <v>7.2604145077720172E-2</v>
-      </c>
-      <c r="Z24" s="20">
+        <v>7.90959585492228</v>
+      </c>
+      <c r="AA24" s="20">
         <f t="shared" si="6"/>
-        <v>7.90959585492228</v>
-      </c>
-      <c r="AA24" s="20">
+        <v>2.0257852979274604</v>
+      </c>
+      <c r="AB24" s="20">
         <f t="shared" si="7"/>
-        <v>2.0257852979274604</v>
-      </c>
-      <c r="AB24" s="20">
-        <f t="shared" si="8"/>
         <v>3.2704569854828905E-2</v>
       </c>
       <c r="AC24" s="20">
@@ -16441,39 +16441,39 @@
         <v>3.0146515695067295</v>
       </c>
       <c r="AD24" s="20">
+        <f t="shared" si="8"/>
+        <v>5.007732297579361</v>
+      </c>
+      <c r="AE24" s="20">
         <f t="shared" si="9"/>
-        <v>5.007732297579361</v>
-      </c>
-      <c r="AE24" s="20">
+        <v>2.9819469996519006</v>
+      </c>
+      <c r="AF24" s="20">
         <f t="shared" si="10"/>
-        <v>2.9819469996519006</v>
-      </c>
-      <c r="AF24" s="20">
+        <v>0.20777285106948312</v>
+      </c>
+      <c r="AG24" s="20">
         <f t="shared" si="11"/>
-        <v>0.20777285106948312</v>
-      </c>
-      <c r="AG24" s="20">
+        <v>0.26226423993417836</v>
+      </c>
+      <c r="AH24" s="20">
         <f t="shared" si="12"/>
-        <v>0.26226423993417836</v>
-      </c>
-      <c r="AH24" s="20">
+        <v>1.9937167976862638</v>
+      </c>
+      <c r="AI24" s="20">
         <f t="shared" si="13"/>
-        <v>1.9937167976862638</v>
-      </c>
-      <c r="AI24" s="20">
+        <v>1.5794765744058687</v>
+      </c>
+      <c r="AJ24" s="20">
         <f t="shared" si="14"/>
-        <v>1.5794765744058687</v>
-      </c>
-      <c r="AJ24" s="20">
+        <v>2.6524937753238444</v>
+      </c>
+      <c r="AK24" s="20">
         <f t="shared" si="15"/>
-        <v>2.6524937753238444</v>
-      </c>
-      <c r="AK24" s="20">
+        <v>0.40453146804726065</v>
+      </c>
+      <c r="AL24" s="20">
         <f t="shared" si="16"/>
-        <v>0.40453146804726065</v>
-      </c>
-      <c r="AL24" s="20">
-        <f t="shared" si="17"/>
         <v>0.67934986710492895</v>
       </c>
     </row>
@@ -16544,7 +16544,7 @@
         <v>7.6215999999999999</v>
       </c>
       <c r="V25" s="20">
-        <f t="shared" si="18"/>
+        <f t="shared" si="17"/>
         <v>10.146999999999998</v>
       </c>
       <c r="W25" s="20">
@@ -16556,19 +16556,19 @@
         <v>1.9978238341968886</v>
       </c>
       <c r="Y25" s="20">
+        <f t="shared" si="18"/>
+        <v>6.9923834196891077E-2</v>
+      </c>
+      <c r="Z25" s="20">
         <f t="shared" si="5"/>
-        <v>6.9923834196891077E-2</v>
-      </c>
-      <c r="Z25" s="20">
+        <v>8.1491761658031105</v>
+      </c>
+      <c r="AA25" s="20">
         <f t="shared" si="6"/>
-        <v>8.1491761658031105</v>
-      </c>
-      <c r="AA25" s="20">
+        <v>1.950999838082899</v>
+      </c>
+      <c r="AB25" s="20">
         <f t="shared" si="7"/>
-        <v>1.950999838082899</v>
-      </c>
-      <c r="AB25" s="20">
-        <f t="shared" si="8"/>
         <v>3.1497222611212197E-2</v>
       </c>
       <c r="AC25" s="20">
@@ -16576,39 +16576,39 @@
         <v>3.1120932735425999</v>
       </c>
       <c r="AD25" s="20">
+        <f t="shared" si="8"/>
+        <v>5.0315958890142873</v>
+      </c>
+      <c r="AE25" s="20">
         <f t="shared" si="9"/>
-        <v>5.0315958890142873</v>
-      </c>
-      <c r="AE25" s="20">
+        <v>3.0805960509313879</v>
+      </c>
+      <c r="AF25" s="20">
         <f t="shared" si="10"/>
-        <v>3.0805960509313879</v>
-      </c>
-      <c r="AF25" s="20">
+        <v>0.1968881279389858</v>
+      </c>
+      <c r="AG25" s="20">
         <f t="shared" si="11"/>
-        <v>0.1968881279389858</v>
-      </c>
-      <c r="AG25" s="20">
+        <v>0.24515654018874689</v>
+      </c>
+      <c r="AH25" s="20">
         <f t="shared" si="12"/>
-        <v>0.24515654018874689</v>
-      </c>
-      <c r="AH25" s="20">
+        <v>2.0166563897061778</v>
+      </c>
+      <c r="AI25" s="20">
         <f t="shared" si="13"/>
-        <v>2.0166563897061778</v>
-      </c>
-      <c r="AI25" s="20">
+        <v>1.6196006884407348</v>
+      </c>
+      <c r="AJ25" s="20">
         <f t="shared" si="14"/>
-        <v>1.6196006884407348</v>
-      </c>
-      <c r="AJ25" s="20">
+        <v>2.6453244862594976</v>
+      </c>
+      <c r="AK25" s="20">
         <f t="shared" si="15"/>
-        <v>2.6453244862594976</v>
-      </c>
-      <c r="AK25" s="20">
+        <v>0.38774970826703431</v>
+      </c>
+      <c r="AL25" s="20">
         <f t="shared" si="16"/>
-        <v>0.38774970826703431</v>
-      </c>
-      <c r="AL25" s="20">
-        <f t="shared" si="17"/>
         <v>0.63331894407026634</v>
       </c>
     </row>
@@ -16679,7 +16679,7 @@
         <v>7.6314000000000002</v>
       </c>
       <c r="V26" s="20">
-        <f t="shared" si="18"/>
+        <f t="shared" si="17"/>
         <v>9.9514999999999976</v>
       </c>
       <c r="W26" s="20">
@@ -16691,19 +16691,19 @@
         <v>1.5119170984455956</v>
       </c>
       <c r="Y26" s="20">
+        <f t="shared" si="18"/>
+        <v>5.2917098445596E-2</v>
+      </c>
+      <c r="Z26" s="20">
         <f t="shared" si="5"/>
-        <v>5.2917098445596E-2</v>
-      </c>
-      <c r="Z26" s="20">
+        <v>8.4395829015544024</v>
+      </c>
+      <c r="AA26" s="20">
         <f t="shared" si="6"/>
-        <v>8.4395829015544024</v>
-      </c>
-      <c r="AA26" s="20">
+        <v>1.476481541450777</v>
+      </c>
+      <c r="AB26" s="20">
         <f t="shared" si="7"/>
-        <v>1.476481541450777</v>
-      </c>
-      <c r="AB26" s="20">
-        <f t="shared" si="8"/>
         <v>2.3836530831349546E-2</v>
       </c>
       <c r="AC26" s="20">
@@ -16711,39 +16711,39 @@
         <v>3.1728798206278004</v>
       </c>
       <c r="AD26" s="20">
+        <f t="shared" si="8"/>
+        <v>4.6255248312472279</v>
+      </c>
+      <c r="AE26" s="20">
         <f t="shared" si="9"/>
-        <v>4.6255248312472279</v>
-      </c>
-      <c r="AE26" s="20">
+        <v>3.1490432897964507</v>
+      </c>
+      <c r="AF26" s="20">
         <f t="shared" si="10"/>
-        <v>3.1490432897964507</v>
-      </c>
-      <c r="AF26" s="20">
+        <v>0.15192856337693775</v>
+      </c>
+      <c r="AG26" s="20">
         <f t="shared" si="11"/>
-        <v>0.15192856337693775</v>
-      </c>
-      <c r="AG26" s="20">
+        <v>0.17914595023020993</v>
+      </c>
+      <c r="AH26" s="20">
         <f t="shared" si="12"/>
-        <v>0.17914595023020993</v>
-      </c>
-      <c r="AH26" s="20">
+        <v>2.1514315376222233</v>
+      </c>
+      <c r="AI26" s="20">
         <f t="shared" si="13"/>
-        <v>2.1514315376222233</v>
-      </c>
-      <c r="AI26" s="20">
+        <v>1.8245676349074427</v>
+      </c>
+      <c r="AJ26" s="20">
         <f t="shared" si="14"/>
-        <v>1.8245676349074427</v>
-      </c>
-      <c r="AJ26" s="20">
+        <v>2.6800466442936464</v>
+      </c>
+      <c r="AK26" s="20">
         <f t="shared" si="15"/>
-        <v>2.6800466442936464</v>
-      </c>
-      <c r="AK26" s="20">
+        <v>0.31920302999490291</v>
+      </c>
+      <c r="AL26" s="20">
         <f t="shared" si="16"/>
-        <v>0.31920302999490291</v>
-      </c>
-      <c r="AL26" s="20">
-        <f t="shared" si="17"/>
         <v>0.46886670190749097</v>
       </c>
     </row>

</xml_diff>